<commit_message>
fix: dual ADF (daily+cumulative), cointegration analysis, economics explanation
</commit_message>
<xml_diff>
--- a/output/tables/factor_model_quality.xlsx
+++ b/output/tables/factor_model_quality.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y26"/>
+  <dimension ref="A1:Z26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -437,22 +437,23 @@
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="26" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
-    <col width="9" customWidth="1" min="12" max="12"/>
-    <col width="8" customWidth="1" min="13" max="13"/>
-    <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="19" customWidth="1" min="15" max="15"/>
-    <col width="13" customWidth="1" min="16" max="16"/>
-    <col width="11" customWidth="1" min="17" max="17"/>
-    <col width="19" customWidth="1" min="18" max="18"/>
-    <col width="13" customWidth="1" min="19" max="19"/>
-    <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="19" customWidth="1" min="21" max="21"/>
-    <col width="13" customWidth="1" min="22" max="22"/>
-    <col width="11" customWidth="1" min="23" max="23"/>
-    <col width="19" customWidth="1" min="24" max="24"/>
-    <col width="13" customWidth="1" min="25" max="25"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="8" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="19" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="11" customWidth="1" min="18" max="18"/>
+    <col width="19" customWidth="1" min="19" max="19"/>
+    <col width="13" customWidth="1" min="20" max="20"/>
+    <col width="11" customWidth="1" min="21" max="21"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="13" customWidth="1" min="23" max="23"/>
+    <col width="11" customWidth="1" min="24" max="24"/>
+    <col width="19" customWidth="1" min="25" max="25"/>
+    <col width="13" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,85 +499,90 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>ADF检验P值</t>
+          <t>ADF(日频残差)P值</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>残差平稳</t>
+          <t>ADF(累积残差)P值</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>累积残差平稳</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>Ljung-Box P值</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>残差白噪声</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>是否通过</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>β_BTC均值</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>β_BTC范围</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>β_BTC变异系数</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>β_QQQ均值</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>β_QQQ范围</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>β_QQQ变异系数</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>β_ETH均值</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>β_ETH范围</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>β_ETH变异系数</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>β_SMH均值</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>β_SMH范围</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>β_SMH变异系数</t>
         </is>
@@ -616,50 +622,53 @@
       <c r="I2" t="n">
         <v>0</v>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" t="n">
+        <v>0.6446</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>0.6739000000000001</v>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="K2" t="n">
-        <v>0.6739000000000001</v>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="n">
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="n">
         <v>0.2795</v>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>[-0.358, 0.690]</t>
         </is>
       </c>
-      <c r="S2" t="n">
+      <c r="T2" t="n">
         <v>0.8129999999999999</v>
       </c>
-      <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr"/>
-      <c r="W2" t="n">
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="n">
         <v>0.9385</v>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="Y2" t="inlineStr">
         <is>
           <t>[0.353, 1.571]</t>
         </is>
       </c>
-      <c r="Y2" t="n">
+      <c r="Z2" t="n">
         <v>0.301</v>
       </c>
     </row>
@@ -697,52 +706,55 @@
       <c r="I3" t="n">
         <v>0</v>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J3" t="n">
+        <v>0.1791</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>0.6317</v>
+      </c>
+      <c r="M3" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="K3" t="n">
-        <v>0.6317</v>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N3" t="n">
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="O3" t="n">
         <v>0.2178</v>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>[-0.277, 0.716]</t>
         </is>
       </c>
-      <c r="P3" t="n">
+      <c r="Q3" t="n">
         <v>1.178</v>
       </c>
-      <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
-      <c r="T3" t="n">
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="n">
         <v>0.9778</v>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="V3" t="inlineStr">
         <is>
           <t>[0.408, 1.526]</t>
         </is>
       </c>
-      <c r="V3" t="n">
+      <c r="W3" t="n">
         <v>0.283</v>
       </c>
-      <c r="W3" t="inlineStr"/>
       <c r="X3" t="inlineStr"/>
       <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -778,52 +790,55 @@
       <c r="I4" t="n">
         <v>0</v>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J4" t="n">
+        <v>0.666</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>0.2619</v>
+      </c>
+      <c r="M4" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="K4" t="n">
-        <v>0.2619</v>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N4" t="n">
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="O4" t="n">
         <v>0.6516999999999999</v>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>[-0.040, 1.277]</t>
         </is>
       </c>
-      <c r="P4" t="n">
+      <c r="Q4" t="n">
         <v>0.361</v>
       </c>
-      <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr"/>
-      <c r="T4" t="n">
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="n">
         <v>0.552</v>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>[0.158, 1.442]</t>
         </is>
       </c>
-      <c r="V4" t="n">
+      <c r="W4" t="n">
         <v>0.456</v>
       </c>
-      <c r="W4" t="inlineStr"/>
       <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -859,52 +874,55 @@
       <c r="I5" t="n">
         <v>3.554660325258204e-30</v>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="K5" t="n">
+      <c r="J5" t="n">
+        <v>0.2025</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
         <v>0.0256</v>
       </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
       <c r="M5" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="N5" t="n">
+      <c r="O5" t="n">
         <v>0.3905</v>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>[-0.474, 0.941]</t>
         </is>
       </c>
-      <c r="P5" t="n">
+      <c r="Q5" t="n">
         <v>0.624</v>
       </c>
-      <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
-      <c r="T5" t="n">
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="n">
         <v>0.7203000000000001</v>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="V5" t="inlineStr">
         <is>
           <t>[0.262, 1.632]</t>
         </is>
       </c>
-      <c r="V5" t="n">
+      <c r="W5" t="n">
         <v>0.39</v>
       </c>
-      <c r="W5" t="inlineStr"/>
       <c r="X5" t="inlineStr"/>
       <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -940,52 +958,55 @@
       <c r="I6" t="n">
         <v>0</v>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J6" t="n">
+        <v>0.441</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>0.8474</v>
+      </c>
+      <c r="M6" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="K6" t="n">
-        <v>0.8474</v>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N6" t="n">
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="O6" t="n">
         <v>0.488</v>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>[0.028, 0.881]</t>
         </is>
       </c>
-      <c r="P6" t="n">
+      <c r="Q6" t="n">
         <v>0.375</v>
       </c>
-      <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
-      <c r="T6" t="n">
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="n">
         <v>0.5848</v>
       </c>
-      <c r="U6" t="inlineStr">
+      <c r="V6" t="inlineStr">
         <is>
           <t>[0.250, 0.959]</t>
         </is>
       </c>
-      <c r="V6" t="n">
+      <c r="W6" t="n">
         <v>0.295</v>
       </c>
-      <c r="W6" t="inlineStr"/>
       <c r="X6" t="inlineStr"/>
       <c r="Y6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1021,52 +1042,55 @@
       <c r="I7" t="n">
         <v>1.047832382721468e-29</v>
       </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="K7" t="n">
+      <c r="J7" t="n">
+        <v>0.1491</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
         <v>0.037</v>
       </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
       <c r="M7" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="N7" t="n">
+      <c r="O7" t="n">
         <v>0.551</v>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>[0.032, 1.111]</t>
         </is>
       </c>
-      <c r="P7" t="n">
+      <c r="Q7" t="n">
         <v>0.384</v>
       </c>
-      <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
-      <c r="T7" t="n">
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="n">
         <v>0.6171</v>
       </c>
-      <c r="U7" t="inlineStr">
+      <c r="V7" t="inlineStr">
         <is>
           <t>[-0.016, 1.099]</t>
         </is>
       </c>
-      <c r="V7" t="n">
+      <c r="W7" t="n">
         <v>0.365</v>
       </c>
-      <c r="W7" t="inlineStr"/>
       <c r="X7" t="inlineStr"/>
       <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1102,52 +1126,55 @@
       <c r="I8" t="n">
         <v>0</v>
       </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="K8" t="n">
+      <c r="J8" t="n">
+        <v>0.2436</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
         <v>0.016</v>
       </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
       <c r="M8" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="N8" t="n">
+      <c r="O8" t="n">
         <v>0.1322</v>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>[-0.449, 0.723]</t>
         </is>
       </c>
-      <c r="P8" t="n">
+      <c r="Q8" t="n">
         <v>2.283</v>
       </c>
-      <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr"/>
-      <c r="T8" t="n">
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="n">
         <v>1.1906</v>
       </c>
-      <c r="U8" t="inlineStr">
+      <c r="V8" t="inlineStr">
         <is>
           <t>[0.661, 1.927]</t>
         </is>
       </c>
-      <c r="V8" t="n">
+      <c r="W8" t="n">
         <v>0.255</v>
       </c>
-      <c r="W8" t="inlineStr"/>
       <c r="X8" t="inlineStr"/>
       <c r="Y8" t="inlineStr"/>
+      <c r="Z8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1183,52 +1210,55 @@
       <c r="I9" t="n">
         <v>0</v>
       </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="K9" t="n">
+      <c r="J9" t="n">
+        <v>0.5021</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
         <v>0.02</v>
       </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
       <c r="M9" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="N9" t="n">
+      <c r="O9" t="n">
         <v>0.2687</v>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="P9" t="inlineStr">
         <is>
           <t>[-0.475, 0.701]</t>
         </is>
       </c>
-      <c r="P9" t="n">
+      <c r="Q9" t="n">
         <v>0.915</v>
       </c>
-      <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr"/>
-      <c r="T9" t="n">
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="n">
         <v>0.8148</v>
       </c>
-      <c r="U9" t="inlineStr">
+      <c r="V9" t="inlineStr">
         <is>
           <t>[0.407, 1.615]</t>
         </is>
       </c>
-      <c r="V9" t="n">
+      <c r="W9" t="n">
         <v>0.341</v>
       </c>
-      <c r="W9" t="inlineStr"/>
       <c r="X9" t="inlineStr"/>
       <c r="Y9" t="inlineStr"/>
+      <c r="Z9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1264,50 +1294,53 @@
       <c r="I10" t="n">
         <v>0</v>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="J10" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
+        <v>0.7211</v>
+      </c>
+      <c r="M10" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="K10" t="n">
-        <v>0.7211</v>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="n">
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="n">
         <v>0.327</v>
       </c>
-      <c r="R10" t="inlineStr">
+      <c r="S10" t="inlineStr">
         <is>
           <t>[-0.343, 0.968]</t>
         </is>
       </c>
-      <c r="S10" t="n">
+      <c r="T10" t="n">
         <v>0.645</v>
       </c>
-      <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr"/>
-      <c r="W10" t="n">
+      <c r="W10" t="inlineStr"/>
+      <c r="X10" t="n">
         <v>0.9510999999999999</v>
       </c>
-      <c r="X10" t="inlineStr">
+      <c r="Y10" t="inlineStr">
         <is>
           <t>[0.457, 1.401]</t>
         </is>
       </c>
-      <c r="Y10" t="n">
+      <c r="Z10" t="n">
         <v>0.26</v>
       </c>
     </row>
@@ -1345,36 +1378,38 @@
       <c r="I11" t="n">
         <v>0</v>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J11" t="n">
+        <v>0.1548</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L11" t="n">
+        <v>0.1809</v>
+      </c>
+      <c r="M11" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="K11" t="n">
-        <v>0.1809</v>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N11" t="n">
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="O11" t="n">
         <v>1.2831</v>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="P11" t="inlineStr">
         <is>
           <t>[0.602, 2.213]</t>
         </is>
       </c>
-      <c r="P11" t="n">
+      <c r="Q11" t="n">
         <v>0.338</v>
       </c>
-      <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr"/>
@@ -1383,6 +1418,7 @@
       <c r="W11" t="inlineStr"/>
       <c r="X11" t="inlineStr"/>
       <c r="Y11" t="inlineStr"/>
+      <c r="Z11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1418,52 +1454,55 @@
       <c r="I12" t="n">
         <v>0</v>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="J12" t="n">
+        <v>0.432</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L12" t="n">
+        <v>0.7817</v>
+      </c>
+      <c r="M12" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="K12" t="n">
-        <v>0.7817</v>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N12" t="n">
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="O12" t="n">
         <v>0.3207</v>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="P12" t="inlineStr">
         <is>
           <t>[0.086, 0.561]</t>
         </is>
       </c>
-      <c r="P12" t="n">
+      <c r="Q12" t="n">
         <v>0.378</v>
       </c>
-      <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr"/>
-      <c r="T12" t="n">
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="n">
         <v>0.3203</v>
       </c>
-      <c r="U12" t="inlineStr">
+      <c r="V12" t="inlineStr">
         <is>
           <t>[0.113, 0.689]</t>
         </is>
       </c>
-      <c r="V12" t="n">
+      <c r="W12" t="n">
         <v>0.35</v>
       </c>
-      <c r="W12" t="inlineStr"/>
       <c r="X12" t="inlineStr"/>
       <c r="Y12" t="inlineStr"/>
+      <c r="Z12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1499,52 +1538,55 @@
       <c r="I13" t="n">
         <v>0</v>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="J13" t="n">
+        <v>0.0167</v>
+      </c>
+      <c r="K13" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="K13" t="n">
+      <c r="L13" t="n">
         <v>0.1091</v>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="N13" t="n">
+      <c r="O13" t="n">
         <v>0.3068</v>
       </c>
-      <c r="O13" t="inlineStr">
+      <c r="P13" t="inlineStr">
         <is>
           <t>[-0.298, 0.954]</t>
         </is>
       </c>
-      <c r="P13" t="n">
+      <c r="Q13" t="n">
         <v>0.862</v>
       </c>
-      <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr"/>
-      <c r="T13" t="n">
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="n">
         <v>0.8001</v>
       </c>
-      <c r="U13" t="inlineStr">
+      <c r="V13" t="inlineStr">
         <is>
           <t>[0.335, 1.416]</t>
         </is>
       </c>
-      <c r="V13" t="n">
+      <c r="W13" t="n">
         <v>0.301</v>
       </c>
-      <c r="W13" t="inlineStr"/>
       <c r="X13" t="inlineStr"/>
       <c r="Y13" t="inlineStr"/>
+      <c r="Z13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1580,52 +1622,55 @@
       <c r="I14" t="n">
         <v>0</v>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="J14" t="n">
+        <v>0.5027</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>0.7139</v>
+      </c>
+      <c r="M14" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="K14" t="n">
-        <v>0.7139</v>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N14" t="n">
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="O14" t="n">
         <v>0.234</v>
       </c>
-      <c r="O14" t="inlineStr">
+      <c r="P14" t="inlineStr">
         <is>
           <t>[-0.999, 1.012]</t>
         </is>
       </c>
-      <c r="P14" t="n">
+      <c r="Q14" t="n">
         <v>1.695</v>
       </c>
-      <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr"/>
-      <c r="T14" t="n">
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="n">
         <v>0.9621</v>
       </c>
-      <c r="U14" t="inlineStr">
+      <c r="V14" t="inlineStr">
         <is>
           <t>[0.215, 1.704]</t>
         </is>
       </c>
-      <c r="V14" t="n">
+      <c r="W14" t="n">
         <v>0.302</v>
       </c>
-      <c r="W14" t="inlineStr"/>
       <c r="X14" t="inlineStr"/>
       <c r="Y14" t="inlineStr"/>
+      <c r="Z14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1661,50 +1706,53 @@
       <c r="I15" t="n">
         <v>0</v>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="J15" t="n">
+        <v>0.0226</v>
+      </c>
+      <c r="K15" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="K15" t="n">
+      <c r="L15" t="n">
         <v>0.5363</v>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="n">
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="n">
         <v>1.2803</v>
       </c>
-      <c r="R15" t="inlineStr">
+      <c r="S15" t="inlineStr">
         <is>
           <t>[0.708, 1.646]</t>
         </is>
       </c>
-      <c r="S15" t="n">
+      <c r="T15" t="n">
         <v>0.167</v>
       </c>
-      <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr"/>
-      <c r="W15" t="n">
+      <c r="W15" t="inlineStr"/>
+      <c r="X15" t="n">
         <v>-0.1291</v>
       </c>
-      <c r="X15" t="inlineStr">
+      <c r="Y15" t="inlineStr">
         <is>
           <t>[-0.387, 0.287]</t>
         </is>
       </c>
-      <c r="Y15" t="n">
+      <c r="Z15" t="n">
         <v>1.258</v>
       </c>
     </row>
@@ -1742,52 +1790,55 @@
       <c r="I16" t="n">
         <v>0</v>
       </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="K16" t="n">
+      <c r="J16" t="n">
+        <v>0.632</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
         <v>7.156387431435858e-05</v>
       </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
       <c r="M16" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="N16" t="n">
+      <c r="O16" t="n">
         <v>1.1258</v>
       </c>
-      <c r="O16" t="inlineStr">
+      <c r="P16" t="inlineStr">
         <is>
           <t>[0.771, 1.566]</t>
         </is>
       </c>
-      <c r="P16" t="n">
+      <c r="Q16" t="n">
         <v>0.178</v>
       </c>
-      <c r="Q16" t="n">
+      <c r="R16" t="n">
         <v>0.7706</v>
       </c>
-      <c r="R16" t="inlineStr">
+      <c r="S16" t="inlineStr">
         <is>
           <t>[0.100, 1.324]</t>
         </is>
       </c>
-      <c r="S16" t="n">
+      <c r="T16" t="n">
         <v>0.444</v>
       </c>
-      <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr"/>
       <c r="X16" t="inlineStr"/>
       <c r="Y16" t="inlineStr"/>
+      <c r="Z16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1823,50 +1874,53 @@
       <c r="I17" t="n">
         <v>6.916997988324113e-30</v>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="J17" t="n">
+        <v>0.206</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L17" t="n">
+        <v>0.0517</v>
+      </c>
+      <c r="M17" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="K17" t="n">
-        <v>0.0517</v>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr"/>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="n">
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="n">
         <v>1.0057</v>
       </c>
-      <c r="R17" t="inlineStr">
+      <c r="S17" t="inlineStr">
         <is>
           <t>[0.703, 1.889]</t>
         </is>
       </c>
-      <c r="S17" t="n">
+      <c r="T17" t="n">
         <v>0.231</v>
       </c>
-      <c r="T17" t="inlineStr"/>
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr"/>
-      <c r="W17" t="n">
+      <c r="W17" t="inlineStr"/>
+      <c r="X17" t="n">
         <v>-0.1426</v>
       </c>
-      <c r="X17" t="inlineStr">
+      <c r="Y17" t="inlineStr">
         <is>
           <t>[-0.732, 0.058]</t>
         </is>
       </c>
-      <c r="Y17" t="n">
+      <c r="Z17" t="n">
         <v>1.096</v>
       </c>
     </row>
@@ -1904,52 +1958,55 @@
       <c r="I18" t="n">
         <v>0</v>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="J18" t="n">
+        <v>0.641</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L18" t="n">
+        <v>0.4749</v>
+      </c>
+      <c r="M18" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="K18" t="n">
-        <v>0.4749</v>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="N18" t="n">
+      <c r="O18" t="n">
         <v>0.4956</v>
       </c>
-      <c r="O18" t="inlineStr">
+      <c r="P18" t="inlineStr">
         <is>
           <t>[0.171, 1.131]</t>
         </is>
       </c>
-      <c r="P18" t="n">
+      <c r="Q18" t="n">
         <v>0.52</v>
       </c>
-      <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr"/>
-      <c r="T18" t="n">
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="n">
         <v>0.3826</v>
       </c>
-      <c r="U18" t="inlineStr">
+      <c r="V18" t="inlineStr">
         <is>
           <t>[0.065, 0.755]</t>
         </is>
       </c>
-      <c r="V18" t="n">
+      <c r="W18" t="n">
         <v>0.361</v>
       </c>
-      <c r="W18" t="inlineStr"/>
       <c r="X18" t="inlineStr"/>
       <c r="Y18" t="inlineStr"/>
+      <c r="Z18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1985,60 +2042,63 @@
       <c r="I19" t="n">
         <v>0</v>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="J19" t="n">
+        <v>0.0963</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
+        <v>0.6698</v>
+      </c>
+      <c r="M19" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="K19" t="n">
-        <v>0.6698</v>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
+      <c r="N19" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="N19" t="n">
+      <c r="O19" t="n">
         <v>0.5517</v>
       </c>
-      <c r="O19" t="inlineStr">
+      <c r="P19" t="inlineStr">
         <is>
           <t>[0.222, 0.881]</t>
         </is>
       </c>
-      <c r="P19" t="n">
+      <c r="Q19" t="n">
         <v>0.299</v>
       </c>
-      <c r="Q19" t="n">
+      <c r="R19" t="n">
         <v>0.9767</v>
       </c>
-      <c r="R19" t="inlineStr">
+      <c r="S19" t="inlineStr">
         <is>
           <t>[0.196, 2.086]</t>
         </is>
       </c>
-      <c r="S19" t="n">
+      <c r="T19" t="n">
         <v>0.452</v>
       </c>
-      <c r="T19" t="n">
+      <c r="U19" t="n">
         <v>0.2551</v>
       </c>
-      <c r="U19" t="inlineStr">
+      <c r="V19" t="inlineStr">
         <is>
           <t>[0.052, 0.539]</t>
         </is>
       </c>
-      <c r="V19" t="n">
+      <c r="W19" t="n">
         <v>0.412</v>
       </c>
-      <c r="W19" t="inlineStr"/>
       <c r="X19" t="inlineStr"/>
       <c r="Y19" t="inlineStr"/>
+      <c r="Z19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2074,50 +2134,53 @@
       <c r="I20" t="n">
         <v>0</v>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="J20" t="n">
+        <v>0.5391</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L20" t="n">
+        <v>0.7439</v>
+      </c>
+      <c r="M20" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="K20" t="n">
-        <v>0.7439</v>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr">
+      <c r="N20" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="n">
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="n">
         <v>1.2438</v>
       </c>
-      <c r="R20" t="inlineStr">
+      <c r="S20" t="inlineStr">
         <is>
           <t>[0.009, 1.900]</t>
         </is>
       </c>
-      <c r="S20" t="n">
+      <c r="T20" t="n">
         <v>0.261</v>
       </c>
-      <c r="T20" t="inlineStr"/>
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr"/>
-      <c r="W20" t="n">
+      <c r="W20" t="inlineStr"/>
+      <c r="X20" t="n">
         <v>-0.09420000000000001</v>
       </c>
-      <c r="X20" t="inlineStr">
+      <c r="Y20" t="inlineStr">
         <is>
           <t>[-0.416, 0.321]</t>
         </is>
       </c>
-      <c r="Y20" t="n">
+      <c r="Z20" t="n">
         <v>1.767</v>
       </c>
     </row>
@@ -2155,50 +2218,53 @@
       <c r="I21" t="n">
         <v>1.584609153937943e-25</v>
       </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="K21" t="n">
+      <c r="J21" t="n">
+        <v>0.3526</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L21" t="n">
         <v>0.0229</v>
       </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
       <c r="M21" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="n">
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="n">
         <v>0.9597</v>
       </c>
-      <c r="R21" t="inlineStr">
+      <c r="S21" t="inlineStr">
         <is>
           <t>[0.566, 1.786]</t>
         </is>
       </c>
-      <c r="S21" t="n">
+      <c r="T21" t="n">
         <v>0.303</v>
       </c>
-      <c r="T21" t="inlineStr"/>
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="inlineStr"/>
-      <c r="W21" t="n">
+      <c r="W21" t="inlineStr"/>
+      <c r="X21" t="n">
         <v>-0.16</v>
       </c>
-      <c r="X21" t="inlineStr">
+      <c r="Y21" t="inlineStr">
         <is>
           <t>[-0.517, 0.091]</t>
         </is>
       </c>
-      <c r="Y21" t="n">
+      <c r="Z21" t="n">
         <v>0.895</v>
       </c>
     </row>
@@ -2236,50 +2302,53 @@
       <c r="I22" t="n">
         <v>0</v>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="J22" t="n">
+        <v>0.4847</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L22" t="n">
+        <v>0.4399</v>
+      </c>
+      <c r="M22" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="K22" t="n">
-        <v>0.4399</v>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
+      <c r="N22" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="n">
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="n">
         <v>1.0952</v>
       </c>
-      <c r="R22" t="inlineStr">
+      <c r="S22" t="inlineStr">
         <is>
           <t>[0.618, 1.594]</t>
         </is>
       </c>
-      <c r="S22" t="n">
+      <c r="T22" t="n">
         <v>0.209</v>
       </c>
-      <c r="T22" t="inlineStr"/>
       <c r="U22" t="inlineStr"/>
       <c r="V22" t="inlineStr"/>
-      <c r="W22" t="n">
+      <c r="W22" t="inlineStr"/>
+      <c r="X22" t="n">
         <v>-0.1245</v>
       </c>
-      <c r="X22" t="inlineStr">
+      <c r="Y22" t="inlineStr">
         <is>
           <t>[-0.374, 0.138]</t>
         </is>
       </c>
-      <c r="Y22" t="n">
+      <c r="Z22" t="n">
         <v>1.217</v>
       </c>
     </row>
@@ -2317,50 +2386,53 @@
       <c r="I23" t="n">
         <v>0</v>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="J23" t="n">
+        <v>0.5396</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L23" t="n">
+        <v>0.3821</v>
+      </c>
+      <c r="M23" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="K23" t="n">
-        <v>0.3821</v>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
+      <c r="N23" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="N23" t="n">
+      <c r="O23" t="n">
         <v>1.1283</v>
       </c>
-      <c r="O23" t="inlineStr">
+      <c r="P23" t="inlineStr">
         <is>
           <t>[0.647, 1.866]</t>
         </is>
       </c>
-      <c r="P23" t="n">
+      <c r="Q23" t="n">
         <v>0.32</v>
       </c>
-      <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="inlineStr"/>
-      <c r="W23" t="n">
+      <c r="W23" t="inlineStr"/>
+      <c r="X23" t="n">
         <v>0.5538999999999999</v>
       </c>
-      <c r="X23" t="inlineStr">
+      <c r="Y23" t="inlineStr">
         <is>
           <t>[0.085, 1.259]</t>
         </is>
       </c>
-      <c r="Y23" t="n">
+      <c r="Z23" t="n">
         <v>0.429</v>
       </c>
     </row>
@@ -2398,50 +2470,53 @@
       <c r="I24" t="n">
         <v>1.848343414409015e-28</v>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="J24" t="n">
+        <v>0.716</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L24" t="n">
+        <v>0.3882</v>
+      </c>
+      <c r="M24" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="K24" t="n">
-        <v>0.3882</v>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
+      <c r="N24" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="N24" t="n">
+      <c r="O24" t="n">
         <v>0.9320000000000001</v>
       </c>
-      <c r="O24" t="inlineStr">
+      <c r="P24" t="inlineStr">
         <is>
           <t>[0.577, 1.563]</t>
         </is>
       </c>
-      <c r="P24" t="n">
+      <c r="Q24" t="n">
         <v>0.327</v>
       </c>
-      <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr"/>
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="inlineStr"/>
-      <c r="W24" t="n">
+      <c r="W24" t="inlineStr"/>
+      <c r="X24" t="n">
         <v>0.6715</v>
       </c>
-      <c r="X24" t="inlineStr">
+      <c r="Y24" t="inlineStr">
         <is>
           <t>[0.191, 1.441]</t>
         </is>
       </c>
-      <c r="Y24" t="n">
+      <c r="Z24" t="n">
         <v>0.476</v>
       </c>
     </row>
@@ -2479,50 +2554,53 @@
       <c r="I25" t="n">
         <v>8.365846541899484e-27</v>
       </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="K25" t="n">
+      <c r="J25" t="n">
+        <v>0.2335</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L25" t="n">
         <v>0.0008</v>
       </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
       <c r="M25" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="N25" t="n">
+      <c r="O25" t="n">
         <v>1.0517</v>
       </c>
-      <c r="O25" t="inlineStr">
+      <c r="P25" t="inlineStr">
         <is>
           <t>[0.667, 1.646]</t>
         </is>
       </c>
-      <c r="P25" t="n">
+      <c r="Q25" t="n">
         <v>0.238</v>
       </c>
-      <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr"/>
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr"/>
       <c r="U25" t="inlineStr"/>
       <c r="V25" t="inlineStr"/>
-      <c r="W25" t="n">
+      <c r="W25" t="inlineStr"/>
+      <c r="X25" t="n">
         <v>0.6041</v>
       </c>
-      <c r="X25" t="inlineStr">
+      <c r="Y25" t="inlineStr">
         <is>
           <t>[0.052, 0.996]</t>
         </is>
       </c>
-      <c r="Y25" t="n">
+      <c r="Z25" t="n">
         <v>0.304</v>
       </c>
     </row>
@@ -2560,50 +2638,53 @@
       <c r="I26" t="n">
         <v>0</v>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="J26" t="n">
+        <v>0.2178</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L26" t="n">
+        <v>0.8983</v>
+      </c>
+      <c r="M26" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="K26" t="n">
-        <v>0.8983</v>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr">
+      <c r="N26" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="n">
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="n">
         <v>1.8089</v>
       </c>
-      <c r="R26" t="inlineStr">
+      <c r="S26" t="inlineStr">
         <is>
           <t>[0.398, 3.208]</t>
         </is>
       </c>
-      <c r="S26" t="n">
+      <c r="T26" t="n">
         <v>0.338</v>
       </c>
-      <c r="T26" t="inlineStr"/>
       <c r="U26" t="inlineStr"/>
       <c r="V26" t="inlineStr"/>
-      <c r="W26" t="n">
+      <c r="W26" t="inlineStr"/>
+      <c r="X26" t="n">
         <v>-0.1482</v>
       </c>
-      <c r="X26" t="inlineStr">
+      <c r="Y26" t="inlineStr">
         <is>
           <t>[-0.828, 0.357]</t>
         </is>
       </c>
-      <c r="Y26" t="n">
+      <c r="Z26" t="n">
         <v>1.862</v>
       </c>
     </row>

</xml_diff>